<commit_message>
Update index to 266 and add 59 new businesses from Game 20-10-2026
Scanned addresses 90-265 (שכונת רחביה) and found 59 verified businesses.
Known businesses database updated from 561 to 620 entries.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ux6ryd78YAefzzubHhHZF
</commit_message>
<xml_diff>
--- a/known_businesses/known_businesses.xlsx
+++ b/known_businesses/known_businesses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G562"/>
+  <dimension ref="A1:G621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -18959,6 +18959,2189 @@
         </is>
       </c>
     </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>שיפוצים מ.ק.</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>עזה 7, ירושלים</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>שיפוצים</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80166911/48570</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>ד"ר במברגר נתן</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>עזה 7, ירושלים</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>רופאי שיניים</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/21526680/46230</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>INSPIRE</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>דרך עזה 32, ירושלים</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>פילאטיס</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/26002961</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>אי.בי.סי.י.ב. בע"מ</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>עזה 24, ירושלים</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>שירותים עסקיים</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80175570/12600</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>כץ דניאל</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>עזה 21, ירושלים</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>צבעים וסיידים</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/19345790/41160</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>ציטה להשקעות ישראל בע"מ</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>סעדיה גאון 16, ירושלים</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>יועצי השקעות</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401C041341706C5E41120112</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>טל רוזן פסיכותרפיה למבוגרים צעירים</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>סעדיה גאון 10, ירושלים</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>פסיכותרפיה</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401D0D1A4370655D4D15071342</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>ברזיל ישראל בית השקעות</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>ככר מגנס 7, ירושלים</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>בתי השקעות</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401C04134077605B48170610</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>פיקר שרון דיאטנית קלינית</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>ככר מגנס 4, ירושלים</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>דיאטנים</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/60134780/12080</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>אלברטו קדרות שימושית</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>ככר מגנס 2, ירושלים</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>קדרות</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80283299/43600</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>גאס השקעות</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>התיבונים 7, ירושלים</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>ניהול תיקי השקעות</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/36811450/14370</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>גייבי מערכות</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>התיבונים 20, ירושלים</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>מערכות מחשוב</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>https://webinfo.co.il/details/130383/%D7%92%D7%99%D7%99%D7%91%D7%99-%D7%9E%D7%A2%D7%A8%D7%9B%D7%95%D7%AA-%D7%91%D7%A2-%D7%9E-511317356</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>גוטמן אלחנן</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>התיבונים 18, ירושלים</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>נגרות</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/נגרים/ירושלים/רחביה</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>טיפול קוגניטיבי התנהגותי cbt ירושלים</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>סעדיה גאון 10, ירושלים</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>פסיכותרפיה</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401D0D1A4370655D4D1206114D</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>גן נעמה</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>הרן 8, ירושלים</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>גני ילדים</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/27147750</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>הדרבוקה</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>הרן 7, ירושלים</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>חנות מוסיקה</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80201518/21100</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>הסוויטה בירושלים</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>הרן 14, ירושלים</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>אירועים</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80030956/15570</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>פלאפל הרצוג</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>הרב הרצוג 59, ירושלים</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>מסעדות מזון מהיר</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/62820160/8450</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>סייפן</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>הרב הרצוג 57, ירושלים</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>שירותי ניהול</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/4D12011540</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>סצמסקי שלום</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>הרב הרצוג 53, ירושלים</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>בית ספר לנהיגה</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401C04134676625F4A140012</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>פרופ' פורת שלמה</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>הרב הרצוג 47, ירושלים</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>אורתופדיה</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>https://www.doctors.co.il/expert/orthopedists/18246630</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>אבן הבונים ב.ב.ז.</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 40, ירושלים</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>בנייה ופיקוח</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>https://www.pusher.li/he/biz/abn-hbvnym-b-b-z-bnyh-vpykvh-ba-m</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>המרתף של אייזיק</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>הקרן הקיימת 41, ירושלים</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>חנות אלכוהול</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/10152047</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>חוויה ברחביה</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>הקליר 20, ירושלים</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>השכרת קורקינטים</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/10149447</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>לאונרדו קליכמן</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>דיסקין 8, ירושלים</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>מספרה</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80185641/630</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>ברודשנדל ליקר ושות'</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>דיסקין 28, ירושלים</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>עו"ד</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80154097/9010118</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>מצבר עד הבית</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 9, ירושלים</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>מצברים</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80214136/31230</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>גל מחשבים</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 34, ירושלים</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>חנות מחשבים</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>https://nons.co.il/provider/%D7%92%D7%9C_%D7%9E%D7%97%D7%A9%D7%91%D7%99%D7%9D</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>עו"ד אורי בן שלמה</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 27, ירושלים</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>עו"ד</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80226843/9010118</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>ד"ר ענת אגרנט מגד</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 27, ירושלים</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>רפואה</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80032151/46290</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>ד"ר סורין מגד</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 36, ירושלים</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>פסיכיאטריה</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>https://www.infomed.co.il/experts/91830</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>אינקו שרותי הנדסה בע"מ</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 26, ירושלים</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>הנדסה</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/17649760/26260</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>אילה וילדמן</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 26, ירושלים</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>רפואה סינית</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/%D7%A8%D7%A4%D7%95%D7%90%D7%94-%D7%A1%D7%99%D7%A0%D7%99%D7%AA/%D7%99%D7%A8%D7%95%D7%A9%D7%9C%D7%99%D7%9D/%D7%A7%D7%98%D7%9E%D7%95%D7%9F</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>פרופ' זלוטניק אבינעם</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 23, ירושלים</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>רפואה פנימית</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>https://www.doctors.co.il/expert/internal-doctors/6057410</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>לטיציה ארועים</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 20, ירושלים</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>הפקת אירועים</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/5709704</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>YBtech Solutions</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 19, ירושלים</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>חנות מחשבים</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>https://nons.co.il/provider/YBtech_Solutions</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>יעקב וטורי דמבו</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 19, ירושלים</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>עו"ד</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80264022/25800</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>3 דרימס</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 18, ירושלים</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>עסקים כלליים</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80221038/23620</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>ארץ התמר-אומנות הגינון</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 18, ירושלים</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>גינון</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80103127/11000</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>סיבירסקי ד"ר און</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 11, ירושלים</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>כירורגיה</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401C04134075655D4A1D041A</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>גיא הרשברג</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 11, ירושלים</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>עסקים כלליים</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80045174/24360</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>אם.ג.אם סאן</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>בנימין מטודלה 13, ירושלים</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>ייעוץ עסקי</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80217667/3510</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>נפתלי ישראלי</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>בן לברט 7, ירושלים</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>פסיכולוגים קליניים</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80152257/40270</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>שמיר אורביטו עדה רחל</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>בן לברט 8, ירושלים</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>עו"ד</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401C041345746C5A491D0D1B</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>ד"ר אהוד חשן</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>בן לברט 3, ירושלים</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>עסקים כלליים</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/35429660/38010</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>סופרי פנחס</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>בן לברט 2, ירושלים</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>מכולת</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/6022010/35760</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>גושן איילת</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>בן לברט 13, ירושלים</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>הומאופתיה</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80005070/40030041</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>עו"ד עומר איילת</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>אפודי 3, ירושלים</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>עו"ד</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80227283/9010104</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>זילברמן אליעזר</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>אלפסי 9, ירושלים</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>רו"ח</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/16448300/46140</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>משכן לבטח בע"מ</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>אלפסי 35, ירושלים</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>שיפוצים</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80314169/48570</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>LE BIJOUTIER</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>אלפסי 37, ירושלים</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>תכשיטים</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401D0D1A4370655D4114041345</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>נוימן ענת</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>אלפסי 3, ירושלים</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>תיווך</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/19715300/32970</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>אפשטיין ושות' משרד עו"ד</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>אלפסי 28, ירושלים</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>עו"ד</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80256202/9010118</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>פינקלשטיין טובה</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>אלפסי 16, ירושלים</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>עו"ד</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80154952/38010</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>אבנת תמר</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>אלפסי 17, ירושלים</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>פסיכולוגים קליניים</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/38841600/40270</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>ד"ר נעמי פינס כהני</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>אלפסי 15, ירושלים</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>פסיכותרפיה</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/26887479</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>קבר יאסון</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>אלפסי 12, ירושלים</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>אטרקציה תיירותית</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/1721440</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>אורן נירה</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>אלחריזי 30, ירושלים</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>מספרה</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/38819680/630</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>סטודיו יאל</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>אלחריזי 26, ירושלים</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>רחביה</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>סטודיו מחול</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>https://yael-jerusalem.co.il/%D7%90%D7%9C%D7%97%D7%A8%D7%99%D7%96%D7%99</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>רוטינה Game 20-10-2026</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update index: 90 → 90 + known businesses (Tavily limit, no addresses scanned)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019dxWuZEvTw3xKZC29AWTtd
</commit_message>
<xml_diff>
--- a/known_businesses/known_businesses.xlsx
+++ b/known_businesses/known_businesses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update index: 90 → 90 (no addresses scanned — Tavily credit exhausted)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YbWQ54djn6byjQYJXcgboM
</commit_message>
<xml_diff>
--- a/known_businesses/known_businesses.xlsx
+++ b/known_businesses/known_businesses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update index: 90 → 90 + known businesses (no change — Tavily credits exhausted)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KDybU8ohspV1oDWHSyBvv7
</commit_message>
<xml_diff>
--- a/known_businesses/known_businesses.xlsx
+++ b/known_businesses/known_businesses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update index: 90 → 90 + known businesses (Tavily credit exhausted — no addresses scanned)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGQiuDgUHNDLCXVQYvTYt1
</commit_message>
<xml_diff>
--- a/known_businesses/known_businesses.xlsx
+++ b/known_businesses/known_businesses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update index: 90 → 90 (Tavily credits exhausted, no addresses scanned) + known businesses
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGQiuAoZMPg4rrfhSEdaTQ
</commit_message>
<xml_diff>
--- a/known_businesses/known_businesses.xlsx
+++ b/known_businesses/known_businesses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update index: 90 → 90 (Tavily credit exhausted, no addresses scanned)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGQiuBY9g48gpXbbGAgRpM
</commit_message>
<xml_diff>
--- a/known_businesses/known_businesses.xlsx
+++ b/known_businesses/known_businesses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update index: 90 → 90 + known businesses (no change — Tavily credit exhausted)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGQiuCMq6EDZVdPLB3eL57
</commit_message>
<xml_diff>
--- a/known_businesses/known_businesses.xlsx
+++ b/known_businesses/known_businesses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="עסקים מוכרים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>